<commit_message>
corrección en plantillas de ingresos devengado y recaudado
</commit_message>
<xml_diff>
--- a/public/CuentasCuentas/Devengado-CuentasCuentasSeguidas.xlsx
+++ b/public/CuentasCuentas/Devengado-CuentasCuentasSeguidas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dmijangos\Documents\SAC-IPE\public\CuentasCuentas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81B00D0B-7D47-42AF-A804-3465D5D7A010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C306C1E-0583-4DFD-A0BB-43949D3854A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
@@ -242,61 +242,61 @@
     <t>VII.1.1 (OTROS INGRESOS Y BENEFICIOS)</t>
   </si>
   <si>
-    <t>8.1.4.4.3.9.9.01.13</t>
-  </si>
-  <si>
-    <t>8.1.2.4.3.9.9.01.13</t>
-  </si>
-  <si>
-    <t>4.3.9.9.01.13</t>
+    <t>8.1.4.4.2.1.2.01.18</t>
+  </si>
+  <si>
+    <t>8.1.2.4.2.1.2.01.18</t>
+  </si>
+  <si>
+    <t>4.2.1.2.01.18</t>
+  </si>
+  <si>
+    <t>1.1.2.2.04.02</t>
+  </si>
+  <si>
+    <t>Por el devengado de ingresos por Rendimientos por cuenta productiva de recursos del Fondo de Aportaciones para el Fortalecimiento de las Entidades Federativas (FAFEF)</t>
+  </si>
+  <si>
+    <t>8.1.4.4.2.1.2.01.19</t>
+  </si>
+  <si>
+    <t>8.1.2.4.2.1.2.01.19</t>
+  </si>
+  <si>
+    <t>4.2.1.2.01.19</t>
+  </si>
+  <si>
+    <t>1.1.2.2.04.03</t>
+  </si>
+  <si>
+    <t>Por el devengado de ingresos por Compensación bancaria de recursos del Fondo de Aportaciones para el Fortalecimiento de las Entidades Federativas (FAFEF)</t>
+  </si>
+  <si>
+    <t>8.1.4.4.3.1.9.01.02</t>
+  </si>
+  <si>
+    <t>8.1.2.4.3.1.9.01.02</t>
+  </si>
+  <si>
+    <t>4.3.1.9.01.02</t>
+  </si>
+  <si>
+    <t>1.1.2.9.02</t>
+  </si>
+  <si>
+    <t>Por el devengado de ingresos por compensación bancaria de recursos propios</t>
+  </si>
+  <si>
+    <t>8.1.4.4.1.7.1.02.02</t>
+  </si>
+  <si>
+    <t>8.1.2.4.1.7.1.02.02</t>
+  </si>
+  <si>
+    <t>4.1.7.1.02.02</t>
   </si>
   <si>
     <t>1.1.2.2.02.13</t>
-  </si>
-  <si>
-    <t>Por el devengado de ingresos por compensación bancaria de recursos propios</t>
-  </si>
-  <si>
-    <t>8.1.4.4.2.1.2.01.18</t>
-  </si>
-  <si>
-    <t>8.1.2.4.2.1.2.01.18</t>
-  </si>
-  <si>
-    <t>4.2.1.2.01.18</t>
-  </si>
-  <si>
-    <t>1.1.2.2.04.02</t>
-  </si>
-  <si>
-    <t>Por el devengado de ingresos por Rendimientos por cuenta productiva de recursos del Fondo de Aportaciones para el Fortalecimiento de las Entidades Federativas (FAFEF)</t>
-  </si>
-  <si>
-    <t>8.1.4.4.2.1.2.01.19</t>
-  </si>
-  <si>
-    <t>8.1.2.4.2.1.2.01.19</t>
-  </si>
-  <si>
-    <t>4.2.1.2.01.19</t>
-  </si>
-  <si>
-    <t>1.1.2.2.04.03</t>
-  </si>
-  <si>
-    <t>Por el devengado de ingresos por Compensación bancaria de recursos del Fondo de Aportaciones para el Fortalecimiento de las Entidades Federativas (FAFEF)</t>
-  </si>
-  <si>
-    <t>8.1.4.4.3.9.9.01.14</t>
-  </si>
-  <si>
-    <t>8.1.2.4.3.9.9.01.14</t>
-  </si>
-  <si>
-    <t>4.3.9.9.01.14</t>
-  </si>
-  <si>
-    <t>1.1.2.2.02.14</t>
   </si>
   <si>
     <t>Por el devengado al realizarse de otros ingresos propios derivados de Comisiones por retención en prestaciones , incluye Impuesto al Valor Agregado. 1 y 2</t>
@@ -329,18 +329,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -355,10 +349,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1961,10 +1954,10 @@
       <c r="A92" t="s">
         <v>68</v>
       </c>
-      <c r="B92" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C92" s="2" t="s">
+      <c r="B92" t="s">
+        <v>67</v>
+      </c>
+      <c r="C92" t="s">
         <v>72</v>
       </c>
       <c r="D92" t="s">

</xml_diff>